<commit_message>
feat: add function to drop components from base data frames
</commit_message>
<xml_diff>
--- a/data/altium_bom.xlsx
+++ b/data/altium_bom.xlsx
@@ -413,109 +413,69 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A5:D36"/>
+  <dimension ref="A7:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="5">
-      <c r="B5" t="inlineStr">
+    <row r="7">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Footprint</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Designator</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>0</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>100K</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>0603</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>R5, R16</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>100K</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>R22</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>100n</t>
+          <t>-5V</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>C23</t>
+          <t>PS1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>100p</t>
+          <t>100K</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>C5, C8, C12, C24</t>
+          <t>R21</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -529,37 +489,37 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>C13, C19</t>
+          <t>C5, C30</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>100uH</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>L1, L4</t>
+          <t>R17, R25</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>10n</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -569,17 +529,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>R6, R13, R18, R19, R25, R27, R29</t>
+          <t>C16</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>10n</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -589,17 +549,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>R1, R10, R14</t>
+          <t>C12, C22</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10n</t>
+          <t>10p</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -609,17 +569,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>C1, C9, C16, C25</t>
+          <t>C3, C14</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10n</t>
+          <t>10p</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -629,17 +589,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>C2, C29</t>
+          <t>C17</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10p</t>
+          <t>10uH</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -649,37 +609,37 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>C4, C10, C21</t>
+          <t>L5</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10p</t>
+          <t>1K</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>C14, C15, C28, C30</t>
+          <t>R19</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10uH</t>
+          <t>1K</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -689,17 +649,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>L2, L3</t>
+          <t>R1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>1u</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -709,17 +669,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>PS3</t>
+          <t>C15, C21</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1K</t>
+          <t>1uH</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -729,77 +689,77 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>R8, R20</t>
+          <t>L4</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1K</t>
+          <t>2200n</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>R7, R21, R24</t>
+          <t>C1, C27</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1u</t>
+          <t>2200n</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>C7, C17</t>
+          <t>C6</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1u</t>
+          <t>220n</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>C18, C20, C27</t>
+          <t>C23, C25, C26</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1uH</t>
+          <t>470</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -809,17 +769,17 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>L5</t>
+          <t>R14</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2200n</t>
+          <t>4K7</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -829,37 +789,37 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>C6, C11</t>
+          <t>R4, R16, R22</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2200n</t>
+          <t>500</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>R3, R5, R9, R24, R27, R29</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>220n</t>
+          <t>500</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -869,187 +829,27 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>C22, C26</t>
+          <t>R13</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>470</t>
+          <t>5K</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>R4</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>23</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>470</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>R3, R17, R26</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>24</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>4K7</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>0603</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>R12, R15</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>25</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>4K7</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>R11, R23</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>26</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>0603</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>27</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>R9, R30</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>28</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>5K</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
           <t>R28</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>29</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>5V</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>0603</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>PS1</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>30</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>9V</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>0603</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>PS2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor:make altium bom sheet index to start at 1
</commit_message>
<xml_diff>
--- a/data/altium_bom.xlsx
+++ b/data/altium_bom.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A7:D28"/>
+  <dimension ref="A7:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="7">
@@ -435,16 +435,16 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>-5V</t>
+          <t>-12V</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -455,7 +455,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -464,22 +464,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>R21</t>
+          <t>R15</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>100p</t>
+          <t>100K</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -489,37 +489,37 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>C5, C30</t>
+          <t>R4</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>100n</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>R17, R25</t>
+          <t>C12</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10n</t>
+          <t>100p</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -529,57 +529,57 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C2, C5, C9, C29</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10n</t>
+          <t>100uH</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>C12, C22</t>
+          <t>L5</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10p</t>
+          <t>100uH</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>C3, C14</t>
+          <t>L3, L4</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10p</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -589,17 +589,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>R2, R28</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10uH</t>
+          <t>10n</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -609,17 +609,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>L5</t>
+          <t>C10, C21, C22</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1K</t>
+          <t>10p</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -629,17 +629,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>R19</t>
+          <t>C15</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1K</t>
+          <t>10p</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -649,37 +649,37 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>C14, C20, C24, C28</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1u</t>
+          <t>10uH</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C15, C21</t>
+          <t>L2</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1uH</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -689,17 +689,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>L4</t>
+          <t>PS2</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2200n</t>
+          <t>1K</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -709,17 +709,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>C1, C27</t>
+          <t>R5, R8, R13, R25, R27</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2200n</t>
+          <t>1K</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -729,17 +729,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>R10, R22, R23</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>220n</t>
+          <t>1u</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -749,17 +749,17 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>C23, C25, C26</t>
+          <t>C6</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>470</t>
+          <t>1u</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -769,37 +769,37 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>R14</t>
+          <t>C1, C7, C13</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>4K7</t>
+          <t>1uH</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>R4, R16, R22</t>
+          <t>L1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>2200n</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -809,17 +809,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>R3, R5, R9, R24, R27, R29</t>
+          <t>C4, C8, C16</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>2200n</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -829,27 +829,187 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>R13</t>
+          <t>C17, C23, C25</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>220n</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>C27, C30</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>22</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>470</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>0603</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>R16, R19, R26</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>23</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>470</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>R1, R29</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>24</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>4K7</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>0603</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>R6, R14</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>25</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>4K7</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>R18</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>26</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>0603</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>R3, R12</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>27</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>R20</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>28</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>5K</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>R28</t>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>0603</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>R11, R24</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>29</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>5V</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>PS3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: change read functions to also manipulate sheets into a desired format
</commit_message>
<xml_diff>
--- a/data/altium_bom.xlsx
+++ b/data/altium_bom.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A7:D36"/>
+  <dimension ref="A7:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="7">
@@ -459,7 +459,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>100K</t>
+          <t>100n</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -469,7 +469,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>R15</t>
+          <t>C2, C14</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>100K</t>
+          <t>100n</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -489,7 +489,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>C8</t>
         </is>
       </c>
     </row>
@@ -499,17 +499,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>100n</t>
+          <t>100p</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>C12</t>
+          <t>C17, C21</t>
         </is>
       </c>
     </row>
@@ -519,17 +519,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>100p</t>
+          <t>100uH</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>C2, C5, C9, C29</t>
+          <t>L1, L4</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>100uH</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>L5</t>
+          <t>R16, R18</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>100uH</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>L3, L4</t>
+          <t>R15</t>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>10p</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>R2, R28</t>
+          <t>C3, C10</t>
         </is>
       </c>
     </row>
@@ -599,17 +599,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10n</t>
+          <t>10uH</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>C10, C21, C22</t>
+          <t>L2</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10p</t>
+          <t>1K</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>C15</t>
+          <t>R1, R4, R19, R29</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10p</t>
+          <t>1K</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>C14, C20, C24, C28</t>
+          <t>R24</t>
         </is>
       </c>
     </row>
@@ -659,17 +659,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10uH</t>
+          <t>1u</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>C15</t>
         </is>
       </c>
     </row>
@@ -679,17 +679,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>1u</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>PS2</t>
+          <t>C4</t>
         </is>
       </c>
     </row>
@@ -699,7 +699,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1K</t>
+          <t>2200n</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>R5, R8, R13, R25, R27</t>
+          <t>C5</t>
         </is>
       </c>
     </row>
@@ -719,7 +719,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1K</t>
+          <t>2200n</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>R10, R22, R23</t>
+          <t>C11, C20, C26</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1u</t>
+          <t>220n</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C29</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1u</t>
+          <t>220n</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>C1, C7, C13</t>
+          <t>C9</t>
         </is>
       </c>
     </row>
@@ -779,17 +779,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1uH</t>
+          <t>470</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>R30</t>
         </is>
       </c>
     </row>
@@ -799,17 +799,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2200n</t>
+          <t>470</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>C4, C8, C16</t>
+          <t>R14, R25</t>
         </is>
       </c>
     </row>
@@ -819,7 +819,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2200n</t>
+          <t>4K7</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>C17, C23, C25</t>
+          <t>R10</t>
         </is>
       </c>
     </row>
@@ -839,17 +839,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>220n</t>
+          <t>500</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>C27, C30</t>
+          <t>R26</t>
         </is>
       </c>
     </row>
@@ -859,17 +859,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>470</t>
+          <t>500</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>R16, R19, R26</t>
+          <t>R22, R23</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>470</t>
+          <t>5K</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>R1, R29</t>
+          <t>R17</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>4K7</t>
+          <t>9V</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -908,106 +908,6 @@
         </is>
       </c>
       <c r="D31" t="inlineStr">
-        <is>
-          <t>R6, R14</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>25</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>4K7</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>R18</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>26</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>0603</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>R3, R12</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>27</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>R20</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>28</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>5K</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>0603</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>R11, R24</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>29</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>5V</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
         <is>
           <t>PS3</t>
         </is>

</xml_diff>